<commit_message>
Add word "forhåbentlig" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:V2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -493,9 +493,77 @@
         <v>Lapses</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>4728145c-846c-4218-a08b-363918d89a7d</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C2" t="str">
+        <v>forhåbentlig</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>-t, -eBøjningsformerforhåbentligtforhåbentlige som adverbium: -t eller -, for eksempel “vi er forhåbentlig(t) enige” Se bøjning i skemaBøjningsformerforhåbentligt eller forhåbentlig</v>
+      </c>
+      <c r="H2" t="str">
+        <v>[fʌˈhɔˀbənli]</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014619_1.mp3</v>
+      </c>
+      <c r="J2" t="str">
+        <v>1. som man håber på vil blive resultatet SPROGBRUG denne brug regnes af nogle for ukorrektFNs børneorganisation UNICEF scorer det forhåbentlige overskud Pol99Politiken (avis), 1999.1.asom adverbium idet man håber at noget sådant vil skeSynonym sjælde</v>
+      </c>
+      <c r="K2" t="str">
+        <v>hopefully</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O2" t="str">
+        <v>https://ing.dk/#:~:text=forh%C3%A5bentlig</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -504,22 +572,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -583,8 +651,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="28.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "nødvendige" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -561,9 +561,77 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>f714ea22-d0bc-4fec-9b02-440a5f41975b</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C3" t="str">
+        <v>nødvendige</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>-t, -eBøjningsformernødvendigtnødvendige -ere, -stBøjningsformernødvendigerenødvendigst</v>
+      </c>
+      <c r="H3" t="str">
+        <v>[nøðˈvεnˀdi]</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://static.ordnet.dk/mp3/11036/11036670_1.mp3</v>
+      </c>
+      <c r="J3" t="str">
+        <v>1. som der absolut er behov for; som er en uomgængelig betingelse eller forudsætningSynonym fornødenOrd i nærhedenuundgåeligikke til at komme udenomuundværliguomgængelignaturnødvendigpåkrævet Henter ... Henter ... Eksemplernødvendige oplysningeren nø</v>
+      </c>
+      <c r="K3" t="str">
+        <v>necessary</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N3" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O3" t="str">
+        <v>https://ing.dk/#:~:text=n%C3%B8dvendige</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "tilretninger" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -629,9 +629,77 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>bfc64d6a-d4cc-4af8-ac60-6804dbb1b4dd</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C4" t="str">
+        <v>tilretninger</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F4" t="str">
+        <v>en</v>
+      </c>
+      <c r="G4" t="str">
+        <v>-en, -er, -erneBøjningsformertilretningentilretningertilretningerne</v>
+      </c>
+      <c r="H4" t="str">
+        <v>[ˈtelˌʁadneŋ]</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://static.ordnet.dk/mp3/51002/51002634_1.mp3</v>
+      </c>
+      <c r="J4" t="str">
+        <v>det at ændre på noget indtil det passer, ser pænt ud, lyder rigtigt el.lign.Ord i nærhedenjusteringafpasningden nødvendige tilpasningbearbejdelsekorrektivmodifikation Henter ... Henter ... Tilretningen af budgettet giver også mulighed for at løse opg</v>
+      </c>
+      <c r="K4" t="str">
+        <v>adjustments</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Som aftalt med Kim på telefon, sender vi dokumenter fredag. Så kan vi gennemgå dem på mødet og forhåbentlig lave de nødvendige tilretninger.</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Mail - David Yiheng - Outlook</v>
+      </c>
+      <c r="N4" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAANLrW6WeUmyuRwvbPuOOS8%3D</v>
+      </c>
+      <c r="O4" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAANLrW6WeUmyuRwvbPuOOS8%3D#:~:text=tilretninger</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "planlægge" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -697,9 +697,77 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2c1d9555-57fb-48e2-9c5c-349f0c430c86</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C5" t="str">
+        <v>planlægge</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>-r, ..lagde, ..lagtBøjningsformerplanlæggerplagdeplagt</v>
+      </c>
+      <c r="H5" t="str">
+        <v>[ˈplæːnˌlεgə]</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://static.ordnet.dk/mp3/11039/11039990_1.mp3</v>
+      </c>
+      <c r="J5" t="str">
+        <v>forberede, fx ved at udarbejde (detaljerede) planer; have i sindeSynonym sjældent planereSe også påtænkeOrd i nærhedenplanere2anlæggelægge antilrettelæggefastlæggeikke overlade noget til tilfældighederne Henter ... Henter ... grammatikNOGEN planlægge</v>
+      </c>
+      <c r="K5" t="str">
+        <v>plan</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Når I har godkendt RFI, sender vi til de valgte firmaer, og begynder at planlægge præsentationsmøder.</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Mail - David Yiheng - Outlook</v>
+      </c>
+      <c r="N5" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAANLrW6WeUmyuRwvbPuOOS8%3D</v>
+      </c>
+      <c r="O5" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAANLrW6WeUmyuRwvbPuOOS8%3D#:~:text=planl%C3%A6gge</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "nåede" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -765,9 +765,77 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>a2af7418-10c9-4e9a-acb1-b659940a889e</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C6" t="str">
+        <v>nåede</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>-r, -ede, -etBøjningsformernårnåedenået</v>
+      </c>
+      <c r="H6" t="str">
+        <v>[ˈnɔˀ]</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://static.ordnet.dk/mp3/11036/11036717_1.mp3</v>
+      </c>
+      <c r="J6" t="str">
+        <v>1. komme eller bevæge sig helt hen tilOrd i nærhedenhave 2 km tilbagekomme fremnå til vejs endenå sit mållægge noget bag sigindhente Henter ... Henter ... grammatikNOGEN/NOGET når +RETNING HJÆLPEVERBUM være NOGEN/NOGET når NOGET HJÆLPEVERBUM haveEkse</v>
+      </c>
+      <c r="K6" t="str">
+        <v>reached</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Så nåede vi det alligevel i dag 😊</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Mail - David Yiheng - Outlook</v>
+      </c>
+      <c r="N6" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D</v>
+      </c>
+      <c r="O6" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D#:~:text=n%C3%A5ede</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "forneden" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -833,9 +833,77 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>11a89ebe-f0b1-4dcb-af91-49824552266a</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C7" t="str">
+        <v>forneden</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v>adverbium</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>[fʌˈneːðən]</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014895_1.mp3</v>
+      </c>
+      <c r="J7" t="str">
+        <v>1. på eller i den nederste del af nogetSynonymer nederstsjældent nedentilAntonym forovenOrd i nærhedennedentilnedadtilnedenfor1hernedenfor Henter ... Henter ... Blomstringen begynder forneden på blomsterstanden Hjemm1992Hjemmet (blad), 1992.Tjek dine</v>
+      </c>
+      <c r="K7" t="str">
+        <v>below</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Se outline af aktiviteter forneden. Bemærk at en del af estimaterne er afhængige af antallet af firmaer der byder, eks. review af ”tilbud”. Estimaterne er baseret på 3 firmaer.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Mail - David Yiheng - Outlook</v>
+      </c>
+      <c r="N7" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D</v>
+      </c>
+      <c r="O7" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D#:~:text=forneden</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Bemærk" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -901,9 +901,77 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>f410b191-c2cb-4ac3-8924-4b8273585b2c</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Bemærk</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>-r, -de, -tBøjningsformerbemærkerbemærkedebemærket</v>
+      </c>
+      <c r="H8" t="str">
+        <v>[beˈmæɐ̯gə]</v>
+      </c>
+      <c r="I8" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004050_1.mp3</v>
+      </c>
+      <c r="J8" t="str">
+        <v xml:space="preserve">1. blive opmærksom på; lægge mærke tilOrd i nærhedenopdagefå øje pålægge mærke tilregistreresansenotere Henter ... Henter ... grammatikNOGEN bemærker (sig) NOGET/at+SÆTNING/hv+SÆTNINGEksemplerværd/vigtigt at bemærkeikke kunne undgå at bemærkebemærke </v>
+      </c>
+      <c r="K8" t="str">
+        <v>Note</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Se outline af aktiviteter forneden. Bemærk at en del af estimaterne er afhængige af antallet af firmaer der byder, eks. review af ”tilbud”. Estimaterne er baseret på 3 firmaer.</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Mail - David Yiheng - Outlook</v>
+      </c>
+      <c r="N8" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D</v>
+      </c>
+      <c r="O8" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D#:~:text=Bem%C3%A6rk</v>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "afhængige" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -969,9 +969,77 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>cd375258-e3e0-4c9c-b05b-cfdadcefeed5</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C9" t="str">
+        <v>afhængige</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>-t, -eBøjningsformerafhængigtafhængige</v>
+      </c>
+      <c r="H9" t="str">
+        <v>[ɑwˈhεŋˀi]</v>
+      </c>
+      <c r="I9" t="str">
+        <v>https://static.ordnet.dk/mp3/11000/11000465_1.mp3</v>
+      </c>
+      <c r="J9" t="str">
+        <v>1. som har meget brug for eller ikke kan undvære noget eller nogen fx økonomisk eller følelsesmæssigtAntonym uafhængigOrd i nærhedenforudsættebetingekrævepåkrævestå og falde mednødvendiggøre Henter ... Henter ... grammatikafhængig af NOGEN/NOGET/at..</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Dependents</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Se outline af aktiviteter forneden. Bemærk at en del af estimaterne er afhængige af antallet af firmaer der byder, eks. review af ”tilbud”. Estimaterne er baseret på 3 firmaer.</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Mail - David Yiheng - Outlook</v>
+      </c>
+      <c r="N9" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D</v>
+      </c>
+      <c r="O9" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D#:~:text=afh%C3%A6ngige</v>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Selvom" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V10"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1037,9 +1037,77 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>e9fc56ae-9468-4a25-8625-c1f4ba8d92a2</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Selvom</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v>konjunktion</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>[ˈsεlˀʌm]</v>
+      </c>
+      <c r="I10" t="str">
+        <v>https://static.ordnet.dk/mp3/11045/11045430_1.mp3</v>
+      </c>
+      <c r="J10" t="str">
+        <v>1. bruges indrømmende: til trods for den kendsgerning atSynonymer skøntgammeldags ihvorvelOrd i nærhedenmen2skønt Henter ... Henter ... Lene går med ind, selvom hun ikke har lyst AnJoha91Anders Johansen: Englebørn. Gyldendal, 1991.Selv om det er et r</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Though</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Selvom det er samlet forneden, tænker jeg at det giver mening at splitte det op i to tilbud:</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Mail - David Yiheng - Outlook</v>
+      </c>
+      <c r="N10" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D</v>
+      </c>
+      <c r="O10" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D#:~:text=Selvom</v>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "samlet" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:V11"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1105,9 +1105,77 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>f6a5d94c-835e-4029-8b2e-6a825a3c6f7b</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C11" t="str">
+        <v>samlet</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v>-r, -de, -tBøjningsformersamlersamledesamlet</v>
+      </c>
+      <c r="H11" t="str">
+        <v>[ˈsɑmlə]</v>
+      </c>
+      <c r="I11" t="str">
+        <v>https://static.ordnet.dk/mp3/11044/11044641_1.mp3</v>
+      </c>
+      <c r="J11" t="str">
+        <v>1. bringe genstande sammen der forekommer spredt, ofte for at udnytte demOrd i nærhedenbundtestablebunke sammenbundle2opstableophobe Henter ... Henter ... grammatikNOGEN samler NOGETEksemplersamle brændesamle stensamle flaskerIvan rejste sig og gav s</v>
+      </c>
+      <c r="K11" t="str">
+        <v>gathered</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Selvom det er samlet forneden, tænker jeg at det giver mening at splitte det op i to tilbud:</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Mail - David Yiheng - Outlook</v>
+      </c>
+      <c r="N11" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D</v>
+      </c>
+      <c r="O11" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D#:~:text=samlet</v>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "giver mening" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -401,28 +401,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V11"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1182,24 +1182,24 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="7.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1252,9 +1252,59 @@
         <v>Lapses</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>21570780-7bb6-4019-99ff-a97ea98ba44a</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C2" t="str">
+        <v>giver mening</v>
+      </c>
+      <c r="D2" t="str">
+        <v>giver=gives · mening=opinion</v>
+      </c>
+      <c r="E2" t="str">
+        <v>makes sense</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Selvom det er samlet forneden, tænker jeg at det giver mening at splitte det op i to tilbud:</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Mail - David Yiheng - Outlook</v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D#:~:text=giver%20mening</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "tilbud" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,30 +399,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V12"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="7.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1173,9 +1173,77 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>b7260653-9c5d-48d2-9c8c-1f631b7a099f</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C12" t="str">
+        <v>tilbud</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F12" t="str">
+        <v>et</v>
+      </c>
+      <c r="G12" t="str">
+        <v>-det (eller uofficiel form: -et), -, -dene (eller uofficiel form: -ene) Se bøjning i skemaBøjningsformertilbuddet (eller uofficiel form: tilbudet)tilbudtilbuddene (eller uofficiel form: tilbudene)Bemæ</v>
+      </c>
+      <c r="H12" t="str">
+        <v>[ˈtelˌbuð]</v>
+      </c>
+      <c r="I12" t="str">
+        <v>https://static.ordnet.dk/mp3/12001/12001073_1.mp3</v>
+      </c>
+      <c r="J12" t="str">
+        <v>1. udsagn hvormed en person tilbyder en anden person nogetOrd i nærhedenovertalelseforslag1lokkemadmaddingfristelsemiddel1gulerod Henter ... Henter ... grammatiktilbud til NOGEN om NOGET/at..Eksemplerfavorabelt tilbudfristende tilbudgenerøst tilbudfå</v>
+      </c>
+      <c r="K12" t="str">
+        <v>offer</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Selvom det er samlet forneden, tænker jeg at det giver mening at splitte det op i to tilbud:</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Mail - David Yiheng - Outlook</v>
+      </c>
+      <c r="N12" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D</v>
+      </c>
+      <c r="O12" t="str">
+        <v>https://outlook.office.com/mail/inbox/id/AAQkADc2ODI5MjBhLWIzMzAtNGY1OC1iZjYzLTNmMGE5MDdiZTU1OAAQAAzF4AYG%2BMlPjSQyIUifyek%3D#:~:text=tilbud</v>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1184,22 +1252,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "øget" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:V13"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1241,9 +1241,77 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>c7c9c14e-6fa4-4281-9ee9-7cba36006292</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C13" t="str">
+        <v>øget</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F13" t="str">
+        <v>et</v>
+      </c>
+      <c r="G13" t="str">
+        <v>-et, -, -eneBøjningsformerøgetøgøgene</v>
+      </c>
+      <c r="H13" t="str">
+        <v>[ˈøˀj]</v>
+      </c>
+      <c r="I13" t="str">
+        <v>https://static.ordnet.dk/mp3/12008/12008194_1.mp3</v>
+      </c>
+      <c r="J13" t="str">
+        <v>gammel, udslidt hest SPROGBRUG nedsættendeSe også krikkeOrd i nærhedenhest Henter ... Henter ... I Eigtveds ridehus på Christiansborg kunne man øve sig på udtjente, stivbenede øg under opsyn af en kongelig berider OWivel86Ole Wivel: Musikken kommer f</v>
+      </c>
+      <c r="K13" t="str">
+        <v>increased</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Seniorerne efterspørger øget fleksibilitet</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Seniorerne efterspørger øget fleksibilitet</v>
+      </c>
+      <c r="N13" t="str">
+        <v>https://ida.dk/om-ida/nyt-fra-ida/debat-seniorerne-efterspoerger-oeget-fleksibilitet</v>
+      </c>
+      <c r="O13" t="str">
+        <v>https://ida.dk/om-ida/nyt-fra-ida/debat-seniorerne-efterspoerger-oeget-fleksibilitet#:~:text=%C3%B8get</v>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "efterspørger" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Arbejde.xlsx
+++ b/12-06-2026-vokab/Arbejde.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ